<commit_message>
Sample row has been added to excel file
</commit_message>
<xml_diff>
--- a/ugur_Ex3A_tables.xlsx
+++ b/ugur_Ex3A_tables.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ceyhunugur/Desktop/yearup docs/DataAnalytics/DATA_Labs/W2_Workshop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE79E5AD-B8EB-5047-893E-6BD582FB26E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F0ABE92-F6FB-A44B-B5D1-C805D30A8D4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4320" yWindow="620" windowWidth="24480" windowHeight="16260" activeTab="2" xr2:uid="{C2ADFAAE-0408-F24E-957C-1F83EEB62217}"/>
+    <workbookView xWindow="4320" yWindow="640" windowWidth="24480" windowHeight="16260" activeTab="3" xr2:uid="{C2ADFAAE-0408-F24E-957C-1F83EEB62217}"/>
   </bookViews>
   <sheets>
     <sheet name="Clients" sheetId="1" r:id="rId1"/>
@@ -42,10 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="23">
-  <si>
-    <t>CREATE TABLE Clients (</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t xml:space="preserve">    client_id INT PRIMARY KEY,</t>
   </si>
@@ -62,9 +59,6 @@
     <t xml:space="preserve">    age INT</t>
   </si>
   <si>
-    <t>);</t>
-  </si>
-  <si>
     <t>Clients</t>
   </si>
   <si>
@@ -111,6 +105,18 @@
   </si>
   <si>
     <t xml:space="preserve">    dog_id INT,</t>
+  </si>
+  <si>
+    <t>Ceyhun Ugur</t>
+  </si>
+  <si>
+    <t>Chicago, IL</t>
+  </si>
+  <si>
+    <t>Bella</t>
+  </si>
+  <si>
+    <t>Golden Retriever</t>
   </si>
 </sst>
 </file>
@@ -158,10 +164,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -496,75 +505,53 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B28773B3-E532-EE40-A3E8-81B41DA7E103}">
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="27.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.33203125" customWidth="1"/>
+    <col min="4" max="5" width="27.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>7</v>
+        <v>5</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="3"/>
+      <c r="B2">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="F9" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="F10" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="F11" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="F12" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="F13" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="F14" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="F15" t="s">
-        <v>6</v>
+      <c r="C2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D2">
+        <v>8478271872</v>
+      </c>
+      <c r="E2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F2">
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -574,41 +561,57 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67F8BC9D-E8A0-3B4D-9953-D5EA1A72A889}">
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="49.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="24.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
+      <c r="D1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A3" s="2" t="s">
+      <c r="E1" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+      <c r="F1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>13</v>
-      </c>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A2" s="3"/>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -617,40 +620,53 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D280870A-9E9C-7F43-B0D2-DC38F3437D83}">
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="29.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="29.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+      <c r="E1" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+      <c r="F1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>18</v>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A2" s="3"/>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" s="4">
+        <v>46093</v>
+      </c>
+      <c r="D2" s="5">
+        <v>0.52083333333333337</v>
+      </c>
+      <c r="E2">
+        <v>45</v>
+      </c>
+      <c r="F2">
+        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -660,26 +676,36 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66E9BD22-C320-8F47-8502-6D9E64B7C9CD}">
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="53.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A3" s="1" t="s">
-        <v>22</v>
-      </c>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" s="3"/>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>